<commit_message>
Cap nhat du an
</commit_message>
<xml_diff>
--- a/backend/app/static/templates/sample_import_template.xlsx
+++ b/backend/app/static/templates/sample_import_template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM3"/>
+  <dimension ref="A1:AN3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
     <col width="50" customWidth="1" min="37" max="37"/>
     <col width="18" customWidth="1" min="38" max="38"/>
     <col width="19" customWidth="1" min="39" max="39"/>
+    <col width="38" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -665,6 +666,11 @@
           <t>shop_name_chinese</t>
         </is>
       </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>listed</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -860,6 +866,11 @@
       <c r="AM2" t="inlineStr">
         <is>
           <t>Shop Trung Quốc</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Trong danh sách (1=import, 0=xóa DB)</t>
         </is>
       </c>
     </row>
@@ -935,19 +946,19 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="V3" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="W3" t="n">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="X3" t="n">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="Y3" t="n">
-        <v>4.92</v>
+        <v>4.84</v>
       </c>
       <c r="Z3" t="n">
         <v>500</v>
@@ -1014,6 +1025,9 @@
         <is>
           <t>示例义乌商行</t>
         </is>
+      </c>
+      <c r="AN3" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>